<commit_message>
Show placeholder coin ranges per recognition type
Deck slide 8 and both submission forms now show indicative coin
ranges; final values to be set by RZM.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gdp8ZePQFTacqXg8dsAmMk
</commit_message>
<xml_diff>
--- a/forms/sbsi-reward-submission-form_2026-09-30.xlsx
+++ b/forms/sbsi-reward-submission-form_2026-09-30.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="139">
   <si>
     <t xml:space="preserve">SBSI REWARD SYSTEM</t>
   </si>
@@ -102,10 +102,10 @@
     <t xml:space="preserve">Period to</t>
   </si>
   <si>
-    <t xml:space="preserve">Proposed Coins</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(credited only after approval)</t>
+    <t xml:space="preserve">Coin Range</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(placeholder; approver sets final coins within the range)</t>
   </si>
   <si>
     <t xml:space="preserve">Achievement Title</t>
@@ -207,6 +207,9 @@
     <t xml:space="preserve">Coins Credited</t>
   </si>
   <si>
+    <t xml:space="preserve">&lt;Within range&gt;</t>
+  </si>
+  <si>
     <t xml:space="preserve">Recorded by (KLC)</t>
   </si>
   <si>
@@ -246,7 +249,7 @@
     <t xml:space="preserve">Measures: Cross-Department Support</t>
   </si>
   <si>
-    <t xml:space="preserve">Coins</t>
+    <t xml:space="preserve">Coin Range (placeholder)</t>
   </si>
   <si>
     <t xml:space="preserve">X</t>
@@ -297,6 +300,9 @@
     <t xml:space="preserve">Spot Award</t>
   </si>
   <si>
+    <t xml:space="preserve">10–20</t>
+  </si>
+  <si>
     <t xml:space="preserve">Permitting</t>
   </si>
   <si>
@@ -324,6 +330,9 @@
     <t xml:space="preserve">Cross-Department Recognition</t>
   </si>
   <si>
+    <t xml:space="preserve">15–30</t>
+  </si>
+  <si>
     <t xml:space="preserve">Interconnection</t>
   </si>
   <si>
@@ -372,6 +381,9 @@
     <t xml:space="preserve">Quality Excellence Award</t>
   </si>
   <si>
+    <t xml:space="preserve">20–40</t>
+  </si>
+  <si>
     <t xml:space="preserve">Project Management</t>
   </si>
   <si>
@@ -405,6 +417,9 @@
     <t xml:space="preserve">Innovation / Process Improvement</t>
   </si>
   <si>
+    <t xml:space="preserve">25–50</t>
+  </si>
+  <si>
     <t xml:space="preserve">Other</t>
   </si>
   <si>
@@ -417,6 +432,9 @@
     <t xml:space="preserve">Employee of the Quarter</t>
   </si>
   <si>
+    <t xml:space="preserve">40–80</t>
+  </si>
+  <si>
     <t xml:space="preserve">Average Handling Time improvement</t>
   </si>
   <si>
@@ -426,7 +444,7 @@
     <t xml:space="preserve">Training &amp; certification programs completed</t>
   </si>
   <si>
-    <t xml:space="preserve">Coin values are proposals from the Performance Qualification Matrix (Reference_Data); RZM to confirm.</t>
+    <t xml:space="preserve">Coin ranges are placeholders; final values will be set by RZM (Reward Criteria).</t>
   </si>
   <si>
     <t xml:space="preserve">Process specifications updated (no delayed sunset reviews)</t>
@@ -548,13 +566,6 @@
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <i val="true"/>
       <sz val="9"/>
       <color rgb="FF595959"/>
@@ -565,6 +576,13 @@
     <font>
       <sz val="8"/>
       <color rgb="FF7F7F7F"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -658,7 +676,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="26">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -743,19 +761,15 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="1" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1699,15 +1713,14 @@
       <c r="B49" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C49" s="21" t="str">
-        <f aca="false">IF($I$48="Approved",$C$17,"")</f>
-        <v/>
-      </c>
-      <c r="D49" s="21"/>
-      <c r="E49" s="21"/>
-      <c r="F49" s="21"/>
+      <c r="C49" s="19" t="s">
+        <v>56</v>
+      </c>
+      <c r="D49" s="19"/>
+      <c r="E49" s="19"/>
+      <c r="F49" s="19"/>
       <c r="H49" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I49" s="20"/>
       <c r="J49" s="20"/>
@@ -1716,7 +1729,7 @@
     </row>
     <row r="50" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B50" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C50" s="20"/>
       <c r="D50" s="20"/>
@@ -1724,47 +1737,47 @@
       <c r="F50" s="20"/>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B52" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="C52" s="22"/>
-      <c r="D52" s="22"/>
-      <c r="E52" s="22"/>
-      <c r="F52" s="22"/>
-      <c r="G52" s="22"/>
-      <c r="H52" s="22"/>
-      <c r="I52" s="22"/>
-      <c r="J52" s="22"/>
-      <c r="K52" s="22"/>
-      <c r="L52" s="22"/>
+      <c r="B52" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="21"/>
+      <c r="D52" s="21"/>
+      <c r="E52" s="21"/>
+      <c r="F52" s="21"/>
+      <c r="G52" s="21"/>
+      <c r="H52" s="21"/>
+      <c r="I52" s="21"/>
+      <c r="J52" s="21"/>
+      <c r="K52" s="21"/>
+      <c r="L52" s="21"/>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B53" s="22"/>
-      <c r="C53" s="22"/>
-      <c r="D53" s="22"/>
-      <c r="E53" s="22"/>
-      <c r="F53" s="22"/>
-      <c r="G53" s="22"/>
-      <c r="H53" s="22"/>
-      <c r="I53" s="22"/>
-      <c r="J53" s="22"/>
-      <c r="K53" s="22"/>
-      <c r="L53" s="22"/>
+      <c r="B53" s="21"/>
+      <c r="C53" s="21"/>
+      <c r="D53" s="21"/>
+      <c r="E53" s="21"/>
+      <c r="F53" s="21"/>
+      <c r="G53" s="21"/>
+      <c r="H53" s="21"/>
+      <c r="I53" s="21"/>
+      <c r="J53" s="21"/>
+      <c r="K53" s="21"/>
+      <c r="L53" s="21"/>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B54" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C54" s="23"/>
-      <c r="D54" s="23"/>
-      <c r="E54" s="23"/>
-      <c r="F54" s="23"/>
-      <c r="G54" s="23"/>
-      <c r="H54" s="23"/>
-      <c r="I54" s="23"/>
-      <c r="J54" s="23"/>
-      <c r="K54" s="23"/>
-      <c r="L54" s="23"/>
+      <c r="B54" s="22" t="s">
+        <v>60</v>
+      </c>
+      <c r="C54" s="22"/>
+      <c r="D54" s="22"/>
+      <c r="E54" s="22"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="22"/>
+      <c r="H54" s="22"/>
+      <c r="I54" s="22"/>
+      <c r="J54" s="22"/>
+      <c r="K54" s="22"/>
+      <c r="L54" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="42">
@@ -1872,299 +1885,299 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="24" t="s">
+      <c r="A1" s="23" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="24" t="s">
+      <c r="B1" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="C1" s="24" t="s">
-        <v>60</v>
-      </c>
-      <c r="D1" s="24" t="s">
+      <c r="C1" s="23" t="s">
         <v>61</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="D1" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="E1" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="G1" s="24" t="s">
+      <c r="F1" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="H1" s="24" t="s">
+      <c r="G1" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="H1" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="J1" s="24" t="s">
+      <c r="I1" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="K1" s="24" t="s">
+      <c r="J1" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="L1" s="24" t="s">
+      <c r="K1" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="L1" s="23" t="s">
         <v>16</v>
       </c>
-      <c r="M1" s="24" t="s">
-        <v>69</v>
+      <c r="M1" s="23" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="25" t="s">
+      <c r="C2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="25" t="s">
+      <c r="D2" s="24" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="25"/>
-      <c r="F2" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="G2" s="25" t="s">
+      <c r="E2" s="24"/>
+      <c r="F2" s="24" t="s">
         <v>71</v>
       </c>
-      <c r="H2" s="25" t="s">
+      <c r="G2" s="24" t="s">
         <v>72</v>
       </c>
-      <c r="I2" s="25" t="s">
+      <c r="H2" s="24" t="s">
         <v>73</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="I2" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="K2" s="25" t="s">
+      <c r="J2" s="24" t="s">
         <v>75</v>
       </c>
-      <c r="L2" s="25" t="s">
+      <c r="K2" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="L2" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="M2" s="25"/>
+      <c r="M2" s="24"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="25" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="25" t="s">
+      <c r="A3" s="24" t="s">
         <v>77</v>
       </c>
-      <c r="C3" s="25" t="s">
+      <c r="B3" s="24" t="s">
         <v>78</v>
       </c>
-      <c r="D3" s="25" t="s">
+      <c r="C3" s="24" t="s">
         <v>79</v>
       </c>
-      <c r="E3" s="25" t="s">
+      <c r="D3" s="24" t="s">
         <v>80</v>
       </c>
-      <c r="G3" s="25" t="s">
+      <c r="E3" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="G3" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="I3" s="25" t="s">
+      <c r="H3" s="24" t="s">
         <v>83</v>
       </c>
-      <c r="J3" s="25" t="s">
+      <c r="I3" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="L3" s="25" t="s">
+      <c r="J3" s="24" t="s">
         <v>85</v>
       </c>
-      <c r="M3" s="25" t="n">
-        <v>10</v>
+      <c r="L3" s="24" t="s">
+        <v>86</v>
+      </c>
+      <c r="M3" s="24" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="25" t="s">
-        <v>86</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>87</v>
-      </c>
-      <c r="C4" s="25" t="s">
+      <c r="A4" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="E4" s="25" t="s">
+      <c r="B4" s="24" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="25" t="s">
+      <c r="C4" s="24" t="s">
         <v>90</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="E4" s="24" t="s">
         <v>91</v>
       </c>
-      <c r="I4" s="25" t="s">
+      <c r="G4" s="24" t="s">
         <v>92</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="H4" s="24" t="s">
         <v>93</v>
       </c>
-      <c r="L4" s="25" t="s">
+      <c r="I4" s="24" t="s">
         <v>94</v>
       </c>
-      <c r="M4" s="25" t="n">
-        <v>15</v>
+      <c r="J4" s="24" t="s">
+        <v>95</v>
+      </c>
+      <c r="L4" s="24" t="s">
+        <v>96</v>
+      </c>
+      <c r="M4" s="24" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="25" t="s">
-        <v>95</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>96</v>
-      </c>
-      <c r="C5" s="25" t="s">
+      <c r="A5" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>99</v>
+      </c>
+      <c r="C5" s="24" t="s">
+        <v>100</v>
+      </c>
+      <c r="G5" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="H5" s="24" t="s">
+        <v>102</v>
+      </c>
+      <c r="I5" s="24" t="s">
+        <v>103</v>
+      </c>
+      <c r="J5" s="24" t="s">
+        <v>104</v>
+      </c>
+      <c r="L5" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="M5" s="24" t="s">
         <v>97</v>
       </c>
-      <c r="G5" s="25" t="s">
-        <v>98</v>
-      </c>
-      <c r="H5" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="I5" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="J5" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="L5" s="25" t="s">
-        <v>102</v>
-      </c>
-      <c r="M5" s="25" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="25" t="s">
-        <v>103</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>104</v>
-      </c>
-      <c r="C6" s="25" t="s">
-        <v>105</v>
-      </c>
-      <c r="G6" s="25" t="s">
+      <c r="A6" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="H6" s="25" t="s">
+      <c r="B6" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="I6" s="25" t="s">
+      <c r="C6" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="J6" s="25" t="s">
+      <c r="G6" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="L6" s="25" t="s">
+      <c r="H6" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="M6" s="25" t="n">
-        <v>20</v>
+      <c r="I6" s="24" t="s">
+        <v>111</v>
+      </c>
+      <c r="J6" s="24" t="s">
+        <v>112</v>
+      </c>
+      <c r="L6" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="M6" s="24" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="25" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>112</v>
-      </c>
-      <c r="C7" s="25" t="s">
-        <v>113</v>
-      </c>
-      <c r="H7" s="25" t="s">
+      <c r="A7" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>116</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>117</v>
+      </c>
+      <c r="H7" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="I7" s="24" t="s">
+        <v>119</v>
+      </c>
+      <c r="J7" s="24" t="s">
+        <v>120</v>
+      </c>
+      <c r="L7" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="M7" s="24" t="s">
         <v>114</v>
       </c>
-      <c r="I7" s="25" t="s">
-        <v>115</v>
-      </c>
-      <c r="J7" s="25" t="s">
-        <v>116</v>
-      </c>
-      <c r="L7" s="25" t="s">
-        <v>117</v>
-      </c>
-      <c r="M7" s="25" t="n">
-        <v>20</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
-        <v>118</v>
-      </c>
-      <c r="H8" s="25" t="s">
-        <v>119</v>
-      </c>
-      <c r="I8" s="25" t="s">
-        <v>120</v>
-      </c>
-      <c r="L8" s="25" t="s">
-        <v>121</v>
-      </c>
-      <c r="M8" s="25" t="n">
-        <v>25</v>
+      <c r="A8" s="24" t="s">
+        <v>122</v>
+      </c>
+      <c r="H8" s="24" t="s">
+        <v>123</v>
+      </c>
+      <c r="I8" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="L8" s="24" t="s">
+        <v>125</v>
+      </c>
+      <c r="M8" s="24" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="25" t="s">
-        <v>122</v>
-      </c>
-      <c r="H9" s="25" t="s">
-        <v>123</v>
-      </c>
-      <c r="I9" s="25" t="s">
-        <v>124</v>
-      </c>
-      <c r="L9" s="25" t="s">
-        <v>125</v>
-      </c>
-      <c r="M9" s="25" t="n">
-        <v>40</v>
+      <c r="A9" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="H9" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="I9" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="L9" s="24" t="s">
+        <v>130</v>
+      </c>
+      <c r="M9" s="24" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H10" s="25" t="s">
-        <v>126</v>
+      <c r="H10" s="24" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H11" s="25" t="s">
-        <v>127</v>
+      <c r="H11" s="24" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H12" s="25" t="s">
-        <v>128</v>
-      </c>
-      <c r="L12" s="26" t="s">
-        <v>129</v>
+      <c r="H12" s="24" t="s">
+        <v>134</v>
+      </c>
+      <c r="L12" s="25" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H13" s="25" t="s">
-        <v>130</v>
+      <c r="H13" s="24" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H14" s="25" t="s">
-        <v>131</v>
+      <c r="H14" s="24" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="H15" s="25" t="s">
-        <v>132</v>
+      <c r="H15" s="24" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>

</xml_diff>